<commit_message>
Update Excel template with professional formatting
</commit_message>
<xml_diff>
--- a/MCFH-Frontend/public/mcfh_template.xlsx
+++ b/MCFH-Frontend/public/mcfh_template.xlsx
@@ -59,7 +59,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="0" formatCode=""/>
   </x:numFmts>
-  <x:fonts count="1">
+  <x:fonts count="2">
     <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
@@ -67,16 +67,29 @@
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF00B4D8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="2">
     <x:border diagonalUp="0" diagonalDown="0">
       <x:left style="none">
         <x:color rgb="FF000000"/>
@@ -94,14 +107,45 @@
         <x:color rgb="FF000000"/>
       </x:diagonal>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFD3D3D3"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD3D3D3"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD3D3D3"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD3D3D3"/>
+      </x:bottom>
+      <x:diagonal style="none">
+        <x:color rgb="FF000000"/>
+      </x:diagonal>
+    </x:border>
   </x:borders>
-  <x:cellStyleXfs count="1">
+  <x:cellStyleXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="1">
+  <x:cellXfs count="3">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -401,53 +445,53 @@
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
   <x:dimension ref="A1:D3"/>
-  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetFormatPr defaultRowHeight="20" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="13.424911" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="38.853482" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="50.710625" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="18.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.139196" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:4">
-      <x:c r="A1" s="0" t="s">
+    <x:row r="1" spans="1:4" ht="20" customHeight="1">
+      <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
+      <x:c r="B1" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C1" s="0" t="s">
+      <x:c r="C1" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D1" s="0" t="s">
+      <x:c r="D1" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:4">
-      <x:c r="A2" s="0" t="s">
+    <x:row r="2" spans="1:4" ht="20" customHeight="1">
+      <x:c r="A2" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B2" s="0" t="s">
+      <x:c r="B2" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C2" s="0" t="s">
+      <x:c r="C2" s="2" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="D2" s="0" t="s">
+      <x:c r="D2" s="2" t="s">
         <x:v>7</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:4">
-      <x:c r="A3" s="0" t="s">
+    <x:row r="3" spans="1:4" ht="20" customHeight="1">
+      <x:c r="A3" s="2" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s">
+      <x:c r="B3" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C3" s="0" t="s">
+      <x:c r="C3" s="2" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D3" s="0" t="s">
+      <x:c r="D3" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
     </x:row>

</xml_diff>